<commit_message>
latest Code Of Rehire Ireland
</commit_message>
<xml_diff>
--- a/Data/Hires/TestDataPoland-Regression.xlsx
+++ b/Data/Hires/TestDataPoland-Regression.xlsx
@@ -1,23 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D86F3EA4-F6A5-4B4C-ABA3-A44FC3246959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase">Sheet1!$A$1:$BY$3</definedName>
   </definedNames>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="137">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -177,11 +191,11 @@
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
         <color theme="1"/>
+        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
@@ -259,307 +273,308 @@
     <t>Test_1</t>
   </si>
   <si>
-    <t>10700288</t>
+    <t>765 Recruitment  (Fihyp Kohawu (10580286))</t>
+  </si>
+  <si>
+    <t>Poland</t>
+  </si>
+  <si>
+    <t>Johnpaul</t>
+  </si>
+  <si>
+    <t>Dickinson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">698 980 460 </t>
+  </si>
+  <si>
+    <t>Landline</t>
+  </si>
+  <si>
+    <t>Home</t>
+  </si>
+  <si>
+    <t>Automation Street Name</t>
+  </si>
+  <si>
+    <t>Greater Poland</t>
+  </si>
+  <si>
+    <t>00001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warsaw  </t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Street Address</t>
+  </si>
+  <si>
+    <t>Test001@gmail.com</t>
+  </si>
+  <si>
+    <t>New Hire</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Permanent</t>
+  </si>
+  <si>
+    <t>Retail Assistant_NEW</t>
+  </si>
+  <si>
+    <t>Part time</t>
+  </si>
+  <si>
+    <t>Za</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RE029_NEW2 </t>
+  </si>
+  <si>
+    <t>5 Days</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Automation Comments here….</t>
+  </si>
+  <si>
+    <t>Open-ended</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>94 Retail Operative</t>
+  </si>
+  <si>
+    <t>01 Accessories</t>
+  </si>
+  <si>
+    <t>0201-Izha</t>
+  </si>
+  <si>
+    <t>Ulga podatkowa obowiązuje</t>
+  </si>
+  <si>
+    <t>1/12 kwoty zmniejszającej podatek</t>
+  </si>
+  <si>
+    <t>Standardowy</t>
+  </si>
+  <si>
+    <t>PESEL</t>
+  </si>
+  <si>
+    <t>Tax ID Number (NIP)</t>
+  </si>
+  <si>
+    <t>Personal Identity (PESEL) Number</t>
+  </si>
+  <si>
+    <t>ID Card</t>
+  </si>
+  <si>
+    <t>SSK456309</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Married (Poland)</t>
+  </si>
+  <si>
+    <t>01/01/2019</t>
+  </si>
+  <si>
+    <t>Citizen (Poland)</t>
+  </si>
+  <si>
+    <t>Bank of Poland</t>
+  </si>
+  <si>
+    <t>NBPLPLPW</t>
+  </si>
+  <si>
+    <t>Checking</t>
+  </si>
+  <si>
+    <t>11111111111111111111111101</t>
+  </si>
+  <si>
+    <t>PL09109024023899695521479863</t>
+  </si>
+  <si>
+    <t>Defaulted</t>
+  </si>
+  <si>
+    <t>Please select a Poland Pay Group</t>
+  </si>
+  <si>
+    <t>PL Monthly</t>
+  </si>
+  <si>
+    <t>Test_2</t>
+  </si>
+  <si>
+    <t>765 Store Management (Kires Pivyba (10226524))</t>
+  </si>
+  <si>
+    <t>Rudy</t>
+  </si>
+  <si>
+    <t>Franecki</t>
+  </si>
+  <si>
+    <t>Auto 25308091</t>
+  </si>
+  <si>
+    <t>Store Manager_NEW</t>
+  </si>
+  <si>
+    <t>Full time</t>
+  </si>
+  <si>
+    <t>RE024_NEW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92 Retail Management </t>
+  </si>
+  <si>
+    <t xml:space="preserve">251 Management Retail </t>
+  </si>
+  <si>
+    <t>SSK456310</t>
   </si>
   <si>
     <t>Passed</t>
-  </si>
-  <si>
-    <t>765 Recruitment  (Fihyp Kohawu (10580286))</t>
-  </si>
-  <si>
-    <t>Poland</t>
-  </si>
-  <si>
-    <t>Narciso</t>
-  </si>
-  <si>
-    <t>Legros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">698 980 460 </t>
-  </si>
-  <si>
-    <t>Landline</t>
-  </si>
-  <si>
-    <t>Home</t>
-  </si>
-  <si>
-    <t>Automation Street Name</t>
-  </si>
-  <si>
-    <t>Greater Poland</t>
-  </si>
-  <si>
-    <t>00001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Warsaw  </t>
-  </si>
-  <si>
-    <t>Test</t>
-  </si>
-  <si>
-    <t>Street Address</t>
-  </si>
-  <si>
-    <t>Test001@gmail.com</t>
-  </si>
-  <si>
-    <t>New Hire</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Permanent</t>
-  </si>
-  <si>
-    <t>Retail Assistant_NEW</t>
-  </si>
-  <si>
-    <t>Part time</t>
-  </si>
-  <si>
-    <t>Za</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RE029_NEW2 </t>
-  </si>
-  <si>
-    <t>5 Days</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>Automation Comments here….</t>
-  </si>
-  <si>
-    <t>Open-ended</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>94 Retail Operative</t>
-  </si>
-  <si>
-    <t>01 Accessories</t>
-  </si>
-  <si>
-    <t>0201-Izha</t>
-  </si>
-  <si>
-    <t>Ulga podatkowa obowiązuje</t>
-  </si>
-  <si>
-    <t>1/12 kwoty zmniejszającej podatek</t>
-  </si>
-  <si>
-    <t>Standardowy</t>
-  </si>
-  <si>
-    <t>PESEL</t>
-  </si>
-  <si>
-    <t>Tax ID Number (NIP)</t>
-  </si>
-  <si>
-    <t>Personal Identity (PESEL) Number</t>
-  </si>
-  <si>
-    <t>ID Card</t>
-  </si>
-  <si>
-    <t>SSK456300</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>Married (Poland)</t>
-  </si>
-  <si>
-    <t>01/01/2019</t>
-  </si>
-  <si>
-    <t>Citizen (Poland)</t>
-  </si>
-  <si>
-    <t>Bank of Poland</t>
-  </si>
-  <si>
-    <t>NBPLPLPW</t>
-  </si>
-  <si>
-    <t>Checking</t>
-  </si>
-  <si>
-    <t>11111111111111111111111101</t>
-  </si>
-  <si>
-    <t>PL09109024023899695521479863</t>
-  </si>
-  <si>
-    <t>Defaulted</t>
-  </si>
-  <si>
-    <t>Please select a Poland Pay Group</t>
-  </si>
-  <si>
-    <t>PL Monthly</t>
-  </si>
-  <si>
-    <t>Test_2</t>
-  </si>
-  <si>
-    <t>765 Store Management (Kires Pivyba (10226524))</t>
-  </si>
-  <si>
-    <t>Trudie</t>
-  </si>
-  <si>
-    <t>Kshlerin</t>
-  </si>
-  <si>
-    <t>Auto 4159077</t>
-  </si>
-  <si>
-    <t>Store Manager_NEW</t>
-  </si>
-  <si>
-    <t>Full time</t>
-  </si>
-  <si>
-    <t>RE024_NEW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">92 Retail Management </t>
-  </si>
-  <si>
-    <t xml:space="preserve">251 Management Retail </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="17" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FFFF0000"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color indexed="8"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color indexed="8"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color indexed="63"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color indexed="12"/>
+      <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color indexed="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <color indexed="8"/>
-      <family val="2"/>
-      <sz val="14"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <color indexed="10"/>
-      <family val="2"/>
-      <sz val="14"/>
-      <name val="Arial"/>
-    </font>
-    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FFFF0000"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <family val="2"/>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
-      <family val="2"/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
-      <family val="2"/>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color indexed="63"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="7"/>
       <color rgb="FF494949"/>
-      <sz val="7"/>
       <name val="Roboto"/>
     </font>
-    <font>
-      <color indexed="63"/>
-      <family val="2"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -568,7 +583,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
+        <fgColor rgb="FFFF0000"/>
       </patternFill>
     </fill>
     <fill>
@@ -591,7 +606,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.7999816888943144"/>
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -605,10 +626,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -618,8 +647,12 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -716,18 +749,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -760,7 +792,7 @@
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -776,7 +808,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -785,6 +817,9 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1065,9 +1100,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BZ5"/>
-  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.81640625" customWidth="1"/>
     <col min="2" max="2" width="156.54296875" customWidth="1"/>
@@ -1139,7 +1174,7 @@
     <col min="78" max="78" width="30.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1" spans="1:78" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:78" s="2" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1375,108 +1410,108 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" ht="35" customHeight="1" spans="1:78" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:78" s="2" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="30" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="52">
+        <v>10700455</v>
+      </c>
+      <c r="C2" s="52" t="s">
+        <v>136</v>
+      </c>
+      <c r="D2" s="31" t="s">
         <v>76</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="E2" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="32" t="s">
+      <c r="F2" s="33" t="s">
         <v>78</v>
       </c>
-      <c r="E2" s="33" t="s">
+      <c r="G2" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="F2" s="34" t="s">
+      <c r="H2" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="G2" s="35" t="s">
+      <c r="I2" s="35" t="s">
         <v>81</v>
       </c>
-      <c r="H2" s="36" t="s">
+      <c r="J2" s="35" t="s">
         <v>82</v>
       </c>
-      <c r="I2" s="36" t="s">
+      <c r="K2" s="36">
+        <v>45705</v>
+      </c>
+      <c r="L2" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="M2" s="35" t="s">
         <v>83</v>
       </c>
-      <c r="J2" s="36" t="s">
+      <c r="N2" s="35" t="s">
         <v>84</v>
       </c>
-      <c r="K2" s="37">
+      <c r="O2" s="35" t="s">
+        <v>85</v>
+      </c>
+      <c r="P2" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q2" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="R2" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="S2" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="T2" s="35" t="s">
+        <v>82</v>
+      </c>
+      <c r="U2" s="35" t="s">
+        <v>88</v>
+      </c>
+      <c r="V2" s="35" t="s">
+        <v>89</v>
+      </c>
+      <c r="W2" s="35" t="s">
+        <v>82</v>
+      </c>
+      <c r="X2" s="37">
         <v>45705</v>
       </c>
-      <c r="L2" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="M2" s="36" t="s">
-        <v>85</v>
-      </c>
-      <c r="N2" s="36" t="s">
-        <v>86</v>
-      </c>
-      <c r="O2" s="36" t="s">
+      <c r="Y2" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z2" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="AA2" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="AB2" s="35" t="s">
+        <v>93</v>
+      </c>
+      <c r="AC2" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="AD2" s="35">
+        <v>765</v>
+      </c>
+      <c r="AE2" s="35" t="s">
+        <v>71</v>
+      </c>
+      <c r="AF2" s="38">
+        <v>10</v>
+      </c>
+      <c r="AG2" s="35" t="s">
         <v>87</v>
       </c>
-      <c r="P2" s="36" t="s">
-        <v>88</v>
-      </c>
-      <c r="Q2" s="36" t="s">
-        <v>89</v>
-      </c>
-      <c r="R2" s="36" t="s">
-        <v>89</v>
-      </c>
-      <c r="S2" s="36" t="s">
-        <v>88</v>
-      </c>
-      <c r="T2" s="36" t="s">
-        <v>84</v>
-      </c>
-      <c r="U2" s="36" t="s">
-        <v>90</v>
-      </c>
-      <c r="V2" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="W2" s="36" t="s">
-        <v>84</v>
-      </c>
-      <c r="X2" s="38">
-        <v>45705</v>
-      </c>
-      <c r="Y2" s="36" t="s">
-        <v>92</v>
-      </c>
-      <c r="Z2" s="36" t="s">
-        <v>93</v>
-      </c>
-      <c r="AA2" s="36" t="s">
-        <v>94</v>
-      </c>
-      <c r="AB2" s="36" t="s">
+      <c r="AH2" s="35" t="s">
         <v>95</v>
-      </c>
-      <c r="AC2" s="36" t="s">
-        <v>96</v>
-      </c>
-      <c r="AD2" s="36">
-        <v>765</v>
-      </c>
-      <c r="AE2" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="AF2" s="39">
-        <v>10</v>
-      </c>
-      <c r="AG2" s="36" t="s">
-        <v>89</v>
-      </c>
-      <c r="AH2" s="36" t="s">
-        <v>97</v>
       </c>
       <c r="AI2" s="18">
         <v>43831</v>
@@ -1484,237 +1519,237 @@
       <c r="AJ2" s="18">
         <v>45293</v>
       </c>
-      <c r="AK2" s="36" t="s">
+      <c r="AK2" s="35" t="s">
+        <v>96</v>
+      </c>
+      <c r="AL2" s="35" t="s">
+        <v>97</v>
+      </c>
+      <c r="AM2" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="AL2" s="36" t="s">
+      <c r="AN2" s="39">
+        <v>110</v>
+      </c>
+      <c r="AO2" s="35" t="s">
         <v>99</v>
       </c>
-      <c r="AM2" s="36" t="s">
+      <c r="AP2" s="35" t="s">
         <v>100</v>
       </c>
-      <c r="AN2" s="40">
+      <c r="AQ2" s="35" t="s">
+        <v>101</v>
+      </c>
+      <c r="AR2" s="40">
+        <v>45705</v>
+      </c>
+      <c r="AS2" s="40">
+        <v>46012</v>
+      </c>
+      <c r="AT2" s="35" t="s">
+        <v>98</v>
+      </c>
+      <c r="AU2" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="AV2" s="32" t="s">
+        <v>103</v>
+      </c>
+      <c r="AW2" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="AX2" s="35" t="s">
+        <v>105</v>
+      </c>
+      <c r="AY2" s="35" t="s">
+        <v>106</v>
+      </c>
+      <c r="AZ2" s="35" t="s">
+        <v>107</v>
+      </c>
+      <c r="BA2" s="35" t="s">
+        <v>108</v>
+      </c>
+      <c r="BB2" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="BC2" s="35" t="s">
+        <v>98</v>
+      </c>
+      <c r="BD2" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="BE2" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="BF2" s="15">
+        <v>9577796953</v>
+      </c>
+      <c r="BG2" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="BH2" s="32" t="s">
         <v>110</v>
       </c>
-      <c r="AO2" s="36" t="s">
-        <v>101</v>
-      </c>
-      <c r="AP2" s="36" t="s">
-        <v>102</v>
-      </c>
-      <c r="AQ2" s="36" t="s">
-        <v>103</v>
-      </c>
-      <c r="AR2" s="41">
-        <v>45705</v>
-      </c>
-      <c r="AS2" s="41">
-        <v>46012</v>
-      </c>
-      <c r="AT2" s="36" t="s">
-        <v>100</v>
-      </c>
-      <c r="AU2" s="36" t="s">
-        <v>104</v>
-      </c>
-      <c r="AV2" s="33" t="s">
-        <v>105</v>
-      </c>
-      <c r="AW2" s="36" t="s">
-        <v>106</v>
-      </c>
-      <c r="AX2" s="36" t="s">
-        <v>107</v>
-      </c>
-      <c r="AY2" s="36" t="s">
-        <v>108</v>
-      </c>
-      <c r="AZ2" s="36" t="s">
-        <v>109</v>
-      </c>
-      <c r="BA2" s="36" t="s">
-        <v>110</v>
-      </c>
-      <c r="BB2" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="BC2" s="36" t="s">
-        <v>100</v>
-      </c>
-      <c r="BD2" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="BE2" s="33" t="s">
+      <c r="BI2" s="15">
+        <v>49778965512</v>
+      </c>
+      <c r="BJ2" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="BK2" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="BF2" s="15">
-        <v>9577796943</v>
-      </c>
-      <c r="BG2" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="BH2" s="33" t="s">
+      <c r="BL2" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="BI2" s="15">
-        <v>49778965501</v>
-      </c>
-      <c r="BJ2" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="BK2" s="36" t="s">
+      <c r="BM2" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="BL2" s="8" t="s">
+      <c r="BN2" s="41">
+        <v>35591</v>
+      </c>
+      <c r="BO2" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="BM2" s="36" t="s">
+      <c r="BP2" s="35" t="s">
         <v>115</v>
       </c>
-      <c r="BN2" s="42">
-        <v>35591</v>
-      </c>
-      <c r="BO2" s="36" t="s">
+      <c r="BQ2" s="35" t="s">
         <v>116</v>
       </c>
-      <c r="BP2" s="36" t="s">
+      <c r="BR2" s="35" t="s">
         <v>117</v>
       </c>
-      <c r="BQ2" s="36" t="s">
+      <c r="BS2" s="42" t="s">
         <v>118</v>
       </c>
-      <c r="BR2" s="36" t="s">
+      <c r="BT2" s="32" t="s">
         <v>119</v>
       </c>
-      <c r="BS2" s="43" t="s">
+      <c r="BU2" s="43" t="s">
         <v>120</v>
       </c>
-      <c r="BT2" s="33" t="s">
+      <c r="BV2" s="43" t="s">
         <v>121</v>
       </c>
-      <c r="BU2" s="44" t="s">
+      <c r="BW2" s="32" t="s">
         <v>122</v>
       </c>
-      <c r="BV2" s="44" t="s">
+      <c r="BX2" s="32" t="s">
         <v>123</v>
       </c>
-      <c r="BW2" s="33" t="s">
+      <c r="BY2" s="32" t="s">
         <v>124</v>
-      </c>
-      <c r="BX2" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="BY2" s="33" t="s">
-        <v>126</v>
       </c>
       <c r="BZ2" s="5">
         <v>40</v>
       </c>
     </row>
-    <row r="3" ht="54" customHeight="1" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:78" ht="54" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" s="44">
+        <v>10700456</v>
+      </c>
+      <c r="C3" s="52" t="s">
+        <v>136</v>
+      </c>
+      <c r="D3" s="31" t="s">
+        <v>126</v>
+      </c>
+      <c r="E3" s="32" t="s">
+        <v>77</v>
+      </c>
+      <c r="F3" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="B3" s="45">
-        <v>10700273</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="G3" s="34" t="s">
+        <v>128</v>
+      </c>
+      <c r="H3" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="I3" s="39" t="s">
+        <v>81</v>
+      </c>
+      <c r="J3" s="39" t="s">
+        <v>82</v>
+      </c>
+      <c r="K3" s="36">
+        <f t="shared" ref="K3" ca="1" si="0">TODAY()-31</f>
+        <v>45843</v>
+      </c>
+      <c r="L3" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="32" t="s">
-        <v>128</v>
-      </c>
-      <c r="E3" s="33" t="s">
-        <v>79</v>
-      </c>
-      <c r="F3" s="34" t="s">
+      <c r="M3" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="N3" s="39" t="s">
+        <v>84</v>
+      </c>
+      <c r="O3" s="45" t="s">
+        <v>85</v>
+      </c>
+      <c r="P3" s="39" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q3" s="39" t="s">
+        <v>87</v>
+      </c>
+      <c r="R3" s="39" t="s">
+        <v>87</v>
+      </c>
+      <c r="S3" s="39" t="s">
+        <v>86</v>
+      </c>
+      <c r="T3" s="39" t="s">
+        <v>82</v>
+      </c>
+      <c r="U3" s="46" t="s">
+        <v>88</v>
+      </c>
+      <c r="V3" s="47" t="s">
+        <v>89</v>
+      </c>
+      <c r="W3" s="39" t="s">
+        <v>82</v>
+      </c>
+      <c r="X3" s="37">
+        <f t="shared" ref="X3" ca="1" si="1">K3</f>
+        <v>45843</v>
+      </c>
+      <c r="Y3" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="Z3" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="G3" s="35" t="s">
+      <c r="AA3" s="48" t="s">
+        <v>92</v>
+      </c>
+      <c r="AB3" s="49" t="s">
         <v>130</v>
       </c>
-      <c r="H3" s="36" t="s">
-        <v>82</v>
-      </c>
-      <c r="I3" s="40" t="s">
-        <v>83</v>
-      </c>
-      <c r="J3" s="40" t="s">
-        <v>84</v>
-      </c>
-      <c r="K3" s="37">
-        <f t="shared" ref="K3" si="0">TODAY()-31</f>
-        <v>45825</v>
-      </c>
-      <c r="L3" s="33" t="s">
-        <v>79</v>
-      </c>
-      <c r="M3" s="33" t="s">
-        <v>85</v>
-      </c>
-      <c r="N3" s="40" t="s">
-        <v>86</v>
-      </c>
-      <c r="O3" s="46" t="s">
-        <v>87</v>
-      </c>
-      <c r="P3" s="40" t="s">
-        <v>88</v>
-      </c>
-      <c r="Q3" s="40" t="s">
-        <v>89</v>
-      </c>
-      <c r="R3" s="40" t="s">
-        <v>89</v>
-      </c>
-      <c r="S3" s="40" t="s">
-        <v>88</v>
-      </c>
-      <c r="T3" s="40" t="s">
-        <v>84</v>
-      </c>
-      <c r="U3" s="47" t="s">
-        <v>90</v>
-      </c>
-      <c r="V3" s="48" t="s">
-        <v>91</v>
-      </c>
-      <c r="W3" s="40" t="s">
-        <v>84</v>
-      </c>
-      <c r="X3" s="38">
-        <f t="shared" ref="X3" si="1">K3</f>
-        <v>45825</v>
-      </c>
-      <c r="Y3" s="36" t="s">
-        <v>92</v>
-      </c>
-      <c r="Z3" s="6" t="s">
+      <c r="AC3" s="48" t="s">
         <v>131</v>
       </c>
-      <c r="AA3" s="49" t="s">
-        <v>94</v>
-      </c>
-      <c r="AB3" s="50" t="s">
-        <v>132</v>
-      </c>
-      <c r="AC3" s="49" t="s">
-        <v>133</v>
-      </c>
-      <c r="AD3" s="51">
+      <c r="AD3" s="50">
         <v>765</v>
       </c>
-      <c r="AE3" s="51" t="s">
+      <c r="AE3" s="50" t="s">
         <v>71</v>
       </c>
       <c r="AF3" s="16">
         <v>40</v>
       </c>
-      <c r="AG3" s="36" t="s">
-        <v>89</v>
-      </c>
-      <c r="AH3" s="36" t="s">
-        <v>97</v>
+      <c r="AG3" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="AH3" s="35" t="s">
+        <v>95</v>
       </c>
       <c r="AI3" s="18">
         <v>43831</v>
@@ -1723,30 +1758,30 @@
         <v>45293</v>
       </c>
       <c r="AK3" s="17" t="s">
-        <v>134</v>
-      </c>
-      <c r="AL3" s="49" t="s">
+        <v>132</v>
+      </c>
+      <c r="AL3" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="AM3" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="AN3" s="39">
+        <v>110</v>
+      </c>
+      <c r="AO3" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="AM3" s="18" t="s">
+      <c r="AP3" s="51" t="s">
         <v>100</v>
       </c>
-      <c r="AN3" s="40">
-        <v>110</v>
-      </c>
-      <c r="AO3" s="40" t="s">
+      <c r="AQ3" s="39" t="s">
         <v>101</v>
       </c>
-      <c r="AP3" s="52" t="s">
-        <v>102</v>
-      </c>
-      <c r="AQ3" s="40" t="s">
-        <v>103</v>
-      </c>
-      <c r="AR3" s="41">
+      <c r="AR3" s="40">
         <v>45705</v>
       </c>
-      <c r="AS3" s="41">
+      <c r="AS3" s="40">
         <v>46012</v>
       </c>
       <c r="AT3" s="20">
@@ -1754,111 +1789,111 @@
         <v>110</v>
       </c>
       <c r="AU3" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="AV3" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="AW3" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="AX3" s="35" t="s">
+        <v>105</v>
+      </c>
+      <c r="AY3" s="35" t="s">
+        <v>106</v>
+      </c>
+      <c r="AZ3" s="35" t="s">
+        <v>107</v>
+      </c>
+      <c r="BA3" s="35" t="s">
+        <v>108</v>
+      </c>
+      <c r="BB3" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="BC3" s="35" t="s">
+        <v>98</v>
+      </c>
+      <c r="BD3" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="BE3" s="32" t="s">
+        <v>109</v>
+      </c>
+      <c r="BF3" s="15">
+        <v>9577796954</v>
+      </c>
+      <c r="BG3" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="BH3" s="32" t="s">
+        <v>110</v>
+      </c>
+      <c r="BI3" s="15">
+        <v>49778965513</v>
+      </c>
+      <c r="BJ3" s="35" t="s">
+        <v>77</v>
+      </c>
+      <c r="BK3" s="35" t="s">
+        <v>111</v>
+      </c>
+      <c r="BL3" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="AV3" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="AW3" s="36" t="s">
-        <v>106</v>
-      </c>
-      <c r="AX3" s="36" t="s">
-        <v>107</v>
-      </c>
-      <c r="AY3" s="36" t="s">
-        <v>108</v>
-      </c>
-      <c r="AZ3" s="36" t="s">
-        <v>109</v>
-      </c>
-      <c r="BA3" s="36" t="s">
-        <v>110</v>
-      </c>
-      <c r="BB3" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="BC3" s="36" t="s">
-        <v>100</v>
-      </c>
-      <c r="BD3" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="BE3" s="33" t="s">
-        <v>111</v>
-      </c>
-      <c r="BF3" s="15">
-        <v>9577796941</v>
-      </c>
-      <c r="BG3" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="BH3" s="33" t="s">
-        <v>112</v>
-      </c>
-      <c r="BI3" s="15">
-        <v>49778965497</v>
-      </c>
-      <c r="BJ3" s="36" t="s">
-        <v>79</v>
-      </c>
-      <c r="BK3" s="36" t="s">
+      <c r="BM3" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="BL3" s="8" t="s">
+      <c r="BN3" s="41">
+        <v>35591</v>
+      </c>
+      <c r="BO3" s="35" t="s">
         <v>114</v>
       </c>
-      <c r="BM3" s="36" t="s">
+      <c r="BP3" s="35" t="s">
         <v>115</v>
       </c>
-      <c r="BN3" s="42">
-        <v>35591</v>
-      </c>
-      <c r="BO3" s="36" t="s">
+      <c r="BQ3" s="35" t="s">
         <v>116</v>
       </c>
-      <c r="BP3" s="36" t="s">
+      <c r="BR3" s="35" t="s">
         <v>117</v>
       </c>
-      <c r="BQ3" s="36" t="s">
+      <c r="BS3" s="42" t="s">
         <v>118</v>
       </c>
-      <c r="BR3" s="36" t="s">
+      <c r="BT3" s="32" t="s">
         <v>119</v>
       </c>
-      <c r="BS3" s="43" t="s">
+      <c r="BU3" s="43" t="s">
         <v>120</v>
       </c>
-      <c r="BT3" s="33" t="s">
+      <c r="BV3" s="43" t="s">
         <v>121</v>
       </c>
-      <c r="BU3" s="44" t="s">
+      <c r="BW3" s="32" t="s">
         <v>122</v>
       </c>
-      <c r="BV3" s="44" t="s">
+      <c r="BX3" s="32" t="s">
         <v>123</v>
       </c>
-      <c r="BW3" s="33" t="s">
+      <c r="BY3" s="32" t="s">
         <v>124</v>
-      </c>
-      <c r="BX3" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="BY3" s="33" t="s">
-        <v>126</v>
       </c>
       <c r="BZ3" s="5">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="27:27" x14ac:dyDescent="0.25">
-      <c r="AA4" s="33"/>
+    <row r="4" spans="1:78" x14ac:dyDescent="0.25">
+      <c r="AA4" s="32"/>
     </row>
-    <row r="5" spans="27:27" x14ac:dyDescent="0.25">
-      <c r="AA5" s="33"/>
+    <row r="5" spans="1:78" x14ac:dyDescent="0.25">
+      <c r="AA5" s="32"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BY3"/>
+  <autoFilter ref="A1:BY3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>